<commit_message>
Updated check logic, added grouping, new test cases.
</commit_message>
<xml_diff>
--- a/rules/CORE-000142/negative/02/data/unit-test-coreid-CG0241-negative 2.xlsx
+++ b/rules/CORE-000142/negative/02/data/unit-test-coreid-CG0241-negative 2.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,6 +110,8 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -588,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -696,12 +698,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>VSELTM</t>
+          <t>VSTPTREF</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-PT4H</t>
+          <t>DOSE</t>
         </is>
       </c>
     </row>
@@ -832,12 +834,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>VSELTM</t>
+          <t>VSTPTREF</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>-PT4H</t>
+          <t>DOSE</t>
         </is>
       </c>
     </row>
@@ -892,386 +894,6 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>VS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>3</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>7</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>VSTPT</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>10MIN POSTDOSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>3</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>7</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>VSTPTNUM</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>3</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>7</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>VSELTM</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>3</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>VISITNUM</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>7</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>VS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>4</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>8</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>VSTPT</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>10MIN POSTDOSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>4</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>8</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>VSTPTNUM</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>4</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>8</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>VSELTM</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>4</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>8</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>VISITNUM</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>4</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>8</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>VS</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>1</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>5</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>VSTPTREF</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>DOSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>6</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>VSTPTREF</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>DOSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>3</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>7</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>VSTPTREF</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>DOSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>4</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>8</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>VSTPTREF</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>DOSE</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1375,7 @@
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>VS</t>
         </is>
@@ -1842,7 +1464,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="X5" s="8" t="inlineStr">
+      <c r="X5" s="11" t="inlineStr">
         <is>
           <t>-PT4H</t>
         </is>
@@ -1943,7 +1565,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="X6" s="8" t="inlineStr">
+      <c r="X6" s="11" t="inlineStr">
         <is>
           <t>-PT4H</t>
         </is>
@@ -1960,7 +1582,7 @@
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>VS</t>
         </is>
@@ -2014,7 +1636,7 @@
       <c r="P7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q7" s="8" t="inlineStr">
+      <c r="Q7" s="11" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -2037,22 +1659,22 @@
       <c r="U7" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="V7" s="8" t="inlineStr">
+      <c r="V7" s="11" t="inlineStr">
         <is>
           <t>10MIN POSTDOSE</t>
         </is>
       </c>
-      <c r="W7" s="8" t="inlineStr">
+      <c r="W7" s="11" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="X7" s="8" t="inlineStr">
+      <c r="X7" s="11" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="Y7" s="9" t="inlineStr">
+      <c r="Y7" s="6" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
@@ -2064,7 +1686,7 @@
           <t>CDISCPILOT01</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>VS</t>
         </is>
@@ -2118,7 +1740,7 @@
       <c r="P8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="Q8" s="8" t="inlineStr">
+      <c r="Q8" s="11" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -2141,22 +1763,22 @@
       <c r="U8" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="V8" s="8" t="inlineStr">
+      <c r="V8" s="11" t="inlineStr">
         <is>
           <t>10MIN POSTDOSE</t>
         </is>
       </c>
-      <c r="W8" s="8" t="inlineStr">
+      <c r="W8" s="11" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="X8" s="8" t="inlineStr">
+      <c r="X8" s="11" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="Y8" s="9" t="inlineStr">
+      <c r="Y8" s="6" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>

</xml_diff>